<commit_message>
Read from excel completed
</commit_message>
<xml_diff>
--- a/Tutorial 7 - Read and Write/Files/Copy of Cities.xlsx
+++ b/Tutorial 7 - Read and Write/Files/Copy of Cities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VB Scripting Course\2026\VBSCourse\Tutorial 7 - Read and Write\Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{75746F34-448C-4B4A-8D64-1CA8F821316B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7DCC998-609B-4D3F-93F2-05ED8EC032D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>